<commit_message>
chore: sync live currency vacancies and english resume routing
</commit_message>
<xml_diff>
--- a/Вакансии_Автопилот_Live.xlsx
+++ b/Вакансии_Автопилот_Live.xlsx
@@ -1316,7 +1316,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>Resume_RU_1.pdf</t>
+          <t>Resume_EN_1.pdf</t>
         </is>
       </c>
       <c r="J13" s="5" t="inlineStr">
@@ -1379,7 +1379,7 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>Resume_RU.pdf</t>
+          <t>Resume_EN.pdf</t>
         </is>
       </c>
       <c r="J14" s="5" t="inlineStr">
@@ -1442,7 +1442,7 @@
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>Resume_RU_1.pdf</t>
+          <t>Resume_EN_1.pdf</t>
         </is>
       </c>
       <c r="J15" s="5" t="inlineStr">

</xml_diff>

<commit_message>
feat: add flagship currency remote resumes (EN/RU) with Klawa V2 microservices architecture and update all resume versions
</commit_message>
<xml_diff>
--- a/Вакансии_Автопилот_Live.xlsx
+++ b/Вакансии_Автопилот_Live.xlsx
@@ -623,7 +623,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Resume_EN_1.pdf</t>
+          <t>Resume_EN_Remote.pdf</t>
         </is>
       </c>
       <c r="J2" s="5" t="inlineStr">
@@ -686,7 +686,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>Resume_EN_1.pdf</t>
+          <t>Resume_EN_Remote.pdf</t>
         </is>
       </c>
       <c r="J3" s="5" t="inlineStr">
@@ -749,7 +749,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Resume_EN_1.pdf</t>
+          <t>Resume_EN_Remote.pdf</t>
         </is>
       </c>
       <c r="J4" s="5" t="inlineStr">
@@ -812,7 +812,7 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Resume_EN_1.pdf</t>
+          <t>Resume_EN_Remote.pdf</t>
         </is>
       </c>
       <c r="J5" s="5" t="inlineStr">
@@ -875,7 +875,7 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Resume_EN_1.pdf</t>
+          <t>Resume_EN_Remote.pdf</t>
         </is>
       </c>
       <c r="J6" s="5" t="inlineStr">
@@ -938,7 +938,7 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>Resume_EN.pdf</t>
+          <t>Resume_EN_Remote.pdf</t>
         </is>
       </c>
       <c r="J7" s="5" t="inlineStr">
@@ -1001,7 +1001,7 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Resume_EN_1.pdf</t>
+          <t>Resume_EN_Remote.pdf</t>
         </is>
       </c>
       <c r="J8" s="5" t="inlineStr">
@@ -1064,7 +1064,7 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>Resume_EN_1.pdf</t>
+          <t>Resume_EN_Remote.pdf</t>
         </is>
       </c>
       <c r="J9" s="5" t="inlineStr">
@@ -1127,7 +1127,7 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Resume_EN.pdf</t>
+          <t>Resume_EN_Remote.pdf</t>
         </is>
       </c>
       <c r="J10" s="5" t="inlineStr">
@@ -1190,7 +1190,7 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>Resume_EN_1.pdf</t>
+          <t>Resume_EN_Remote.pdf</t>
         </is>
       </c>
       <c r="J11" s="5" t="inlineStr">
@@ -1253,7 +1253,7 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>Resume_EN_1.pdf</t>
+          <t>Resume_EN_Remote.pdf</t>
         </is>
       </c>
       <c r="J12" s="5" t="inlineStr">
@@ -1316,7 +1316,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>Resume_EN_1.pdf</t>
+          <t>Resume_EN_Remote.pdf</t>
         </is>
       </c>
       <c r="J13" s="5" t="inlineStr">
@@ -1442,7 +1442,7 @@
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>Resume_EN_1.pdf</t>
+          <t>Resume_EN_Remote.pdf</t>
         </is>
       </c>
       <c r="J15" s="5" t="inlineStr">
@@ -1505,7 +1505,7 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>Resume_EN_1.pdf</t>
+          <t>Resume_EN_Remote.pdf</t>
         </is>
       </c>
       <c r="J16" s="5" t="inlineStr">
@@ -1568,7 +1568,7 @@
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>Resume_EN_1.pdf</t>
+          <t>Resume_EN_Remote.pdf</t>
         </is>
       </c>
       <c r="J17" s="5" t="inlineStr">
@@ -1631,7 +1631,7 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>Resume_EN_1.pdf</t>
+          <t>Resume_EN_Remote.pdf</t>
         </is>
       </c>
       <c r="J18" s="5" t="inlineStr">
@@ -1694,7 +1694,7 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>Resume_EN_1.pdf</t>
+          <t>Resume_EN_Remote.pdf</t>
         </is>
       </c>
       <c r="J19" s="5" t="inlineStr">
@@ -1757,7 +1757,7 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>Resume_EN_1.pdf</t>
+          <t>Resume_EN_Remote.pdf</t>
         </is>
       </c>
       <c r="J20" s="5" t="inlineStr">
@@ -1824,7 +1824,7 @@
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>Resume_EN_1.pdf</t>
+          <t>Resume_EN_Remote.pdf</t>
         </is>
       </c>
       <c r="J21" s="5" t="inlineStr">
@@ -1890,7 +1890,7 @@
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>Resume_EN.pdf</t>
+          <t>Resume_EN_Remote.pdf</t>
         </is>
       </c>
       <c r="J22" s="5" t="inlineStr">
@@ -1957,7 +1957,7 @@
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>Resume_EN_1.pdf</t>
+          <t>Resume_EN_Remote.pdf</t>
         </is>
       </c>
       <c r="J23" s="5" t="inlineStr">
@@ -2025,7 +2025,7 @@
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>Resume_EN_1.pdf</t>
+          <t>Resume_EN_Remote.pdf</t>
         </is>
       </c>
       <c r="J24" s="5" t="inlineStr">
@@ -2090,7 +2090,7 @@
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>Resume_EN_1.pdf</t>
+          <t>Resume_EN_Remote.pdf</t>
         </is>
       </c>
       <c r="J25" s="5" t="inlineStr">
@@ -2153,7 +2153,7 @@
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>Resume_EN_1.pdf</t>
+          <t>Resume_EN_Remote.pdf</t>
         </is>
       </c>
       <c r="J26" s="5" t="inlineStr">
@@ -2216,7 +2216,7 @@
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>Resume_EN_1.pdf</t>
+          <t>Resume_EN_Remote.pdf</t>
         </is>
       </c>
       <c r="J27" s="5" t="inlineStr">
@@ -2279,7 +2279,7 @@
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>Resume_EN_1.pdf</t>
+          <t>Resume_EN_Remote.pdf</t>
         </is>
       </c>
       <c r="J28" s="5" t="inlineStr">
@@ -2342,7 +2342,7 @@
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>Resume_EN.pdf</t>
+          <t>Resume_EN_Remote.pdf</t>
         </is>
       </c>
       <c r="J29" s="5" t="inlineStr">

</xml_diff>